<commit_message>
feat(q3): add exact multiplayer solver foundation
</commit_message>
<xml_diff>
--- a/q1/Result.xlsx
+++ b/q1/Result.xlsx
@@ -555,15 +555,9 @@
       <c r="B4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>178</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>333</v>
-      </c>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
       <c r="G4" s="4" t="n">
         <v>0</v>
       </c>
@@ -584,18 +578,10 @@
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>321</v>
-      </c>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
       <c r="G5" s="4" t="n">
         <v>1</v>
       </c>
@@ -616,18 +602,10 @@
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>146</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>309</v>
-      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
       <c r="G6" s="4" t="n">
         <v>2</v>
       </c>
@@ -648,18 +626,10 @@
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>136</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>295</v>
-      </c>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
       <c r="G7" s="4" t="n">
         <v>3</v>
       </c>
@@ -680,18 +650,10 @@
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>126</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>285</v>
-      </c>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
       <c r="G8" s="4" t="n">
         <v>4</v>
       </c>
@@ -712,18 +674,10 @@
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>116</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>271</v>
-      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
       <c r="G9" s="4" t="n">
         <v>5</v>
       </c>
@@ -744,18 +698,10 @@
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>259</v>
-      </c>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
       <c r="G10" s="4" t="n">
         <v>6</v>
       </c>
@@ -776,18 +722,10 @@
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>90</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>249</v>
-      </c>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
       <c r="G11" s="4" t="n">
         <v>7</v>
       </c>
@@ -808,18 +746,10 @@
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>5780</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>235</v>
-      </c>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
       <c r="G12" s="4" t="n">
         <v>8</v>
       </c>
@@ -840,18 +770,10 @@
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>4150</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>227</v>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>223</v>
-      </c>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
       <c r="G13" s="4" t="n">
         <v>9</v>
       </c>
@@ -872,18 +794,10 @@
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>4150</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>211</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>211</v>
-      </c>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
       <c r="G14" s="4" t="n">
         <v>10</v>
       </c>
@@ -904,18 +818,10 @@
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>5150</v>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>181</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>181</v>
-      </c>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
       <c r="G15" s="4" t="n">
         <v>11</v>
       </c>
@@ -936,18 +842,10 @@
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>6150</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>157</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>163</v>
-      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
       <c r="G16" s="4" t="n">
         <v>12</v>
       </c>
@@ -968,18 +866,10 @@
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>7150</v>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>142</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>142</v>
-      </c>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
       <c r="G17" s="4" t="n">
         <v>13</v>
       </c>
@@ -1000,18 +890,10 @@
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>8150</v>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>118</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>124</v>
-      </c>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
       <c r="G18" s="4" t="n">
         <v>14</v>
       </c>
@@ -1032,18 +914,10 @@
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>9150</v>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>94</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>106</v>
-      </c>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
       <c r="G19" s="4" t="n">
         <v>15</v>
       </c>
@@ -1064,18 +938,10 @@
       <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>10150</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>88</v>
-      </c>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
       <c r="G20" s="4" t="n">
         <v>16</v>
       </c>
@@ -1096,18 +962,10 @@
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>10150</v>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>78</v>
-      </c>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
       <c r="G21" s="4" t="n">
         <v>17</v>
       </c>
@@ -1128,18 +986,10 @@
       <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>10150</v>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>68</v>
-      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
       <c r="G22" s="4" t="n">
         <v>18</v>
       </c>
@@ -1160,18 +1010,10 @@
       <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C23" s="4" t="n">
-        <v>11150</v>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>50</v>
-      </c>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
       <c r="G23" s="4" t="n">
         <v>19</v>
       </c>
@@ -1192,18 +1034,10 @@
       <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>11150</v>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>38</v>
-      </c>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
       <c r="G24" s="4" t="n">
         <v>20</v>
       </c>
@@ -1224,18 +1058,10 @@
       <c r="A25" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="C25" s="4" t="n">
-        <v>11150</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>24</v>
-      </c>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
       <c r="G25" s="4" t="n">
         <v>21</v>
       </c>
@@ -1256,18 +1082,10 @@
       <c r="A26" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>10470</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>26</v>
-      </c>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
       <c r="G26" s="4" t="n">
         <v>22</v>
       </c>
@@ -1288,18 +1106,10 @@
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>10470</v>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>14</v>
-      </c>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
       <c r="G27" s="4" t="n">
         <v>23</v>
       </c>
@@ -1320,18 +1130,10 @@
       <c r="A28" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>10470</v>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>0</v>
-      </c>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
       <c r="G28" s="4" t="n">
         <v>24</v>
       </c>

</xml_diff>